<commit_message>
Remove S&P website URL from GRQDs (org kept, link removed)
</commit_message>
<xml_diff>
--- a/data/raw/landscape-current.xlsx
+++ b/data/raw/landscape-current.xlsx
@@ -2133,11 +2133,7 @@
           <t>Group on Reference Quality Data sets (GRQDs)</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>https://www.spglobal.com/</t>
-        </is>
-      </c>
+      <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
           <t>Focuses on identifying, prioritizing, and preserving “reference-quality” datasets that underpin climate science and key downstream products. The group develops strategies to safeguard high-value, long-term observational records at risk of degradation or loss.</t>

</xml_diff>